<commit_message>
login api spec added to customer page
</commit_message>
<xml_diff>
--- a/Planning/customerAPI.xlsx
+++ b/Planning/customerAPI.xlsx
@@ -1,13 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\IITB_sem1\cs699_softwareLab\Course_project\Apna-Companion\Planning\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3719282F-45F3-4A81-B5D1-EE0473B277CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="login_page" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -18,9 +24,212 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="26">
+  <si>
+    <t>API endpoint</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Request</t>
+  </si>
+  <si>
+    <t>Response</t>
+  </si>
+  <si>
+    <t>SNO</t>
+  </si>
+  <si>
+    <t>auth/login</t>
+  </si>
+  <si>
+    <t>post</t>
+  </si>
+  <si>
+    <t>{
+  "mobile": "+919876543210",
+  "password": "secret123"
+}</t>
+  </si>
+  <si>
+    <t>auth/sendOTP</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OTP service need to be integrated to send OTP to user mobile number and validate it in backend </t>
+  </si>
+  <si>
+    <t>auth/verifyOTP</t>
+  </si>
+  <si>
+    <t>auth/register</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">{
+  "verification_token": "vt_8f3a...",
+  "name": "Rahul Shah",
+  "password": "secret123",
+  "dob": "1995-04-12",
+  "location": "Mumbai"
+} 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Need to decide which all fields is required to take from user during register</t>
+    </r>
+  </si>
+  <si>
+    <t>auth/forgetPassword</t>
+  </si>
+  <si>
+    <t>{
+  "mobile": "+919876543210",
+  "purpose": "PasswordReset"
+}</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">{
+  "mobile": "+919876543210",
+  "purpose": </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>"register" / "passwordReset"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+}</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">{
+  "mobile": "+919876543210",
+  "otp": "482913",
+  "purpose": </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>"register" / "passwordReset"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+}</t>
+    </r>
+  </si>
+  <si>
+    <t>Based on password reset we will open screen to reset password and proceed with further screen</t>
+  </si>
+  <si>
+    <t>auth/setNewPassword</t>
+  </si>
+  <si>
+    <t>{
+  "status_code": 200,
+  "data": {
+    "access_token": "eyJ...",
+    "user": {
+      "id": 12,
+      "name": "Rahul Shah",
+      "mobile": "+919876543210"
+    }
+  }
+}</t>
+  </si>
+  <si>
+    <t>{
+  "status_code": 200,
+  "data": {
+     "expires_in": 300,
+     "resend_after": 30
+    }
+  }
+}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{
+  "status_code": 200,
+  "data": {
+      "expires_in": 300,
+     "resend_after": 30
+  }
+}
+</t>
+  </si>
+  <si>
+    <t>{
+  "status_code": 200,
+  "data": {
+      "verification_token": "vt_8f3a...",
+      "expires_in": 600
+       "purpose": "register" / "passwordReset"
+  }
+}</t>
+  </si>
+  <si>
+    <t>{
+  "status_code": 200,
+  "data": {
+         "message": "successful"
+  }
+}</t>
+  </si>
+  <si>
+    <t>{
+  "status_code": 200,
+  "data": {
+     "message" : "password changed successfully!"
+  }
+}</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -28,16 +237,38 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,12 +276,72 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -330,10 +621,160 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:G7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="9" style="4" customWidth="1"/>
+    <col min="2" max="2" width="34.77734375" style="13" customWidth="1"/>
+    <col min="3" max="3" width="26.21875" style="10" customWidth="1"/>
+    <col min="4" max="4" width="26.77734375" style="10" customWidth="1"/>
+    <col min="5" max="5" width="46.6640625" style="7" customWidth="1"/>
+    <col min="6" max="6" width="41.44140625" style="7" customWidth="1"/>
+    <col min="7" max="7" width="35.5546875" style="15" customWidth="1"/>
+    <col min="8" max="16384" width="8.88671875" style="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" s="1" customFormat="1" ht="18" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="G1" s="5"/>
+    </row>
+    <row r="2" spans="1:7" s="3" customFormat="1" ht="174" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="12"/>
+      <c r="C2" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="G2" s="14"/>
+    </row>
+    <row r="3" spans="1:7" s="3" customFormat="1" ht="174" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="2">
+        <v>2</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="G3" s="14"/>
+    </row>
+    <row r="4" spans="1:7" s="3" customFormat="1" ht="174" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="2">
+        <v>3</v>
+      </c>
+      <c r="B4" s="12"/>
+      <c r="C4" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="G4" s="14" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" s="3" customFormat="1" ht="174" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="2">
+        <v>4</v>
+      </c>
+      <c r="B5" s="12"/>
+      <c r="C5" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="G5" s="14"/>
+    </row>
+    <row r="6" spans="1:7" s="3" customFormat="1" ht="174" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="2">
+        <v>5</v>
+      </c>
+      <c r="B6" s="12"/>
+      <c r="C6" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="G6" s="14"/>
+    </row>
+    <row r="7" spans="1:7" s="3" customFormat="1" ht="174" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="2">
+        <v>6</v>
+      </c>
+      <c r="B7" s="12"/>
+      <c r="C7" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="G7" s="14"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
customer landing page api added
</commit_message>
<xml_diff>
--- a/Planning/customerAPI.xlsx
+++ b/Planning/customerAPI.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\IITB_sem1\cs699_softwareLab\Course_project\Apna-Companion\Planning\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3719282F-45F3-4A81-B5D1-EE0473B277CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21BC81FF-5F55-43F9-B959-B3E0F8020136}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="login_page" sheetId="1" r:id="rId1"/>
+    <sheet name="customer_landingPage" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="47">
   <si>
     <t>API endpoint</t>
   </si>
@@ -64,32 +65,6 @@
   </si>
   <si>
     <t>auth/verifyOTP</t>
-  </si>
-  <si>
-    <t>auth/register</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">{
-  "verification_token": "vt_8f3a...",
-  "name": "Rahul Shah",
-  "password": "secret123",
-  "dob": "1995-04-12",
-  "location": "Mumbai"
-} 
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Need to decide which all fields is required to take from user during register</t>
-    </r>
   </si>
   <si>
     <t>auth/forgetPassword</t>
@@ -169,19 +144,6 @@
     <t>{
   "status_code": 200,
   "data": {
-    "access_token": "eyJ...",
-    "user": {
-      "id": 12,
-      "name": "Rahul Shah",
-      "mobile": "+919876543210"
-    }
-  }
-}</t>
-  </si>
-  <si>
-    <t>{
-  "status_code": 200,
-  "data": {
      "expires_in": 300,
      "resend_after": 30
     }
@@ -224,12 +186,300 @@
   }
 }</t>
   </si>
+  <si>
+    <t>{
+  "userID": "Mobile / Email",
+   "accessToken": ""
+}</t>
+  </si>
+  <si>
+    <t>customer/getBookingDetails</t>
+  </si>
+  <si>
+    <t>For current and past bookings</t>
+  </si>
+  <si>
+    <t>Arrays of booking history</t>
+  </si>
+  <si>
+    <t>customer/getUserInfo</t>
+  </si>
+  <si>
+    <t>customer/getClientDetails</t>
+  </si>
+  <si>
+    <t>{
+  "userID": "Mobile / Email",
+   "accessToken": "",
+   "category": "",
+    "purpose"  : "" 
+}</t>
+  </si>
+  <si>
+    <t>customer/saveBookingDetails</t>
+  </si>
+  <si>
+    <t>{
+  "success": 200,
+  "data": {
+    [
+      { 
+        "id": "pr_12", 
+        "name": "Sunrise Multispeciality Hospital"
+         "costPerHour" : ""
+      },
+      { 
+        "id": "pr_12", 
+        "name": "Sunrise Multispeciality Hospital"
+         "costPerHour" : ""
+      },
+  ],..........
+}</t>
+  </si>
+  <si>
+    <t>{
+  "success": 200,
+  "data": {
+        "message" : "booking confirmed"
+  }
+}</t>
+  </si>
+  <si>
+    <t>customer/saveAddressDetails</t>
+  </si>
+  <si>
+    <t>{
+  "success": 200,
+  "data": {
+        "message" : "Address added"
+  }
+}</t>
+  </si>
+  <si>
+    <t>{
+  "userID": "Mobile / Email",
+  "accessToken": "",
+  "city" :
+  "state" :
+  "pincode" :
+  "address" : "",
+  "addressCatetory" : "",
+  "" : "",
+  "" : "",
+  "" : "",
+}</t>
+  </si>
+  <si>
+    <t>customer/getCurrentBookingDetails</t>
+  </si>
+  <si>
+    <t>{
+  "success": 200,
+  "data": {
+    [
+      "bookingId": "",
+      "status": "completed/rejected",
+      "service": "OPD visit companion",
+      "provider": { 
+        "id": "pr_12", 
+        "name": "Sunrise Multispeciality Hospital"
+      },
+      "companion": { 
+        "name": "Priya S.", 
+        "photo_url": "...",
+        "phone_masked": "+91 98xxxxxx21",
+        "rating": 4.8 
+      },
+      "scheduled_at": "2026-10-17T10:30:00+05:30",
+      "Duration": ,
+      "customer rating": // incase of completed
+      "customer comments": //incase of completed
+    }
+  ],..........
+}</t>
+  </si>
+  <si>
+    <t>{
+  "success": 200,
+  "data": {
+      "bookingId": "",
+      "status": "pending",
+      "estimated_distance": 12, //min
+      "service": "OPD visit companion",
+      "provider": { 
+        "id": "pr_12", 
+        "name": "Sunrise Multispeciality Hospital"
+      },
+      "companion": { 
+        "name": "Priya S.", 
+        "photo_url": "...",
+        "phone_masked": "+91 98xxxxxx21",
+        "rating": 4.8 
+      },
+      "scheduled_at": "2026-10-17T10:30:00+05:30",
+      "Duration": ,
+      "startOtp": ""
+       "endOtp" : ""
+    }
+}</t>
+  </si>
+  <si>
+    <t>{
+  "success": 200,
+  "data": {
+      "userId": "",
+      "mobile_number" : ,
+      "EmailId" : 
+      "full_name" : 
+      "dob":
+      "gender" :
+    }
+}</t>
+  </si>
+  <si>
+    <t>customer/getAddressDetails</t>
+  </si>
+  <si>
+    <t>{
+  "userID": "Mobile / Email",
+  "accessToken": "",
+ }</t>
+  </si>
+  <si>
+    <t>{
+  "success": 200,
+  "data": {
+    [
+      {
+        "city" :
+        "state" :
+        "pincode" :
+        "address" : ""
+        "addressType":""
+      }
+  ],..........
+}</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">{
+  "userID": "Mobile / Email",
+  "accessToken": "",
+   </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>"addressId" : ""</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+  "category": "",
+  "purpose"  : "",
+  "city" :
+  "state" :
+  "pincode" :
+  "address" : "",
+  "timeOfBooking" : "",
+  "durationOfBooking" : "",
+  "dateOfBooking" : "",
+  "additionalComment" : "",
+}</t>
+    </r>
+  </si>
+  <si>
+    <t>auth/saveOrEditUser</t>
+  </si>
+  <si>
+    <t>{
+  "status_code": 200,
+  "data": {
+    "access_token": "eyJ...",
+    "userId": "",
+      "mobile_number" : ,
+      "EmailId" : 
+      "full_name" : 
+      "dob":
+      "gender" :
+      "password" : ""
+  }
+}</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">{
+     "verification_token": "vt_8f3a...",
+     "name": "Rahul Shah",
+     </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>"userId": "",</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+     "mobile_number" : ,
+      "EmailId" : 
+      "full_name" : 
+      "dob":
+      "gender" :
+       </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>"password" : ""  //if enpty ignore</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+} </t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -249,6 +499,13 @@
       <b/>
       <sz val="14"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -295,7 +552,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -341,6 +598,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -671,7 +931,7 @@
         <v>7</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="G2" s="14"/>
     </row>
@@ -689,10 +949,10 @@
         <v>6</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="G3" s="14"/>
     </row>
@@ -708,13 +968,13 @@
         <v>6</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="G4" s="14" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:7" s="3" customFormat="1" ht="174" customHeight="1" x14ac:dyDescent="0.3">
@@ -723,16 +983,16 @@
       </c>
       <c r="B5" s="12"/>
       <c r="C5" s="9" t="s">
-        <v>12</v>
+        <v>44</v>
       </c>
       <c r="D5" s="9" t="s">
         <v>6</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>13</v>
+        <v>46</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="G5" s="14"/>
     </row>
@@ -742,16 +1002,16 @@
       </c>
       <c r="B6" s="12"/>
       <c r="C6" s="9" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D6" s="9" t="s">
         <v>6</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="G6" s="14"/>
     </row>
@@ -761,7 +1021,7 @@
       </c>
       <c r="B7" s="12"/>
       <c r="C7" s="9" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D7" s="9" t="s">
         <v>6</v>
@@ -770,9 +1030,188 @@
         <v>7</v>
       </c>
       <c r="F7" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="G7" s="14"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9CE83456-D14C-4ACF-903E-6FCA1A55BDA8}">
+  <dimension ref="A1:G8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="9" customWidth="1"/>
+    <col min="2" max="2" width="34.77734375" customWidth="1"/>
+    <col min="3" max="3" width="26.21875" style="16" customWidth="1"/>
+    <col min="4" max="4" width="26.77734375" customWidth="1"/>
+    <col min="5" max="5" width="46.6640625" customWidth="1"/>
+    <col min="6" max="6" width="47" customWidth="1"/>
+    <col min="7" max="7" width="35.5546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="18" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="G1" s="5"/>
+    </row>
+    <row r="2" spans="1:7" ht="158.4" x14ac:dyDescent="0.3">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="G2" s="14"/>
+    </row>
+    <row r="3" spans="1:7" ht="345.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="2">
+        <v>2</v>
+      </c>
+      <c r="B3" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="G7" s="14"/>
+      <c r="C3" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="G3" s="14" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="230.4" x14ac:dyDescent="0.3">
+      <c r="A4" s="2">
+        <v>3</v>
+      </c>
+      <c r="B4" s="12"/>
+      <c r="C4" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="G4" s="14"/>
+    </row>
+    <row r="5" spans="1:7" ht="216" x14ac:dyDescent="0.3">
+      <c r="A5" s="2">
+        <v>4</v>
+      </c>
+      <c r="B5" s="12"/>
+      <c r="C5" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="G5" s="14"/>
+    </row>
+    <row r="6" spans="1:7" ht="172.8" x14ac:dyDescent="0.3">
+      <c r="A6" s="2">
+        <v>4</v>
+      </c>
+      <c r="B6" s="12"/>
+      <c r="C6" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="G6" s="14"/>
+    </row>
+    <row r="7" spans="1:7" ht="331.2" x14ac:dyDescent="0.3">
+      <c r="A7" s="2">
+        <v>5</v>
+      </c>
+      <c r="B7" s="12"/>
+      <c r="C7" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="G7" s="14" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="216" x14ac:dyDescent="0.3">
+      <c r="A8" s="2">
+        <v>4</v>
+      </c>
+      <c r="B8" s="12"/>
+      <c r="C8" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="G8" s="14"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>